<commit_message>
add a new model
</commit_message>
<xml_diff>
--- a/s10.xlsx
+++ b/s10.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20366"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\py_xw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\py_xw\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFCEB9D2-BE12-43EF-9C85-BE8F520FDD26}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20955" windowHeight="7125" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20955" windowHeight="7125" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="星" sheetId="1" r:id="rId1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="784">
   <si>
     <t>首字母</t>
   </si>
@@ -2630,11 +2631,499 @@
 E：二轨条</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>A152</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：滑球后让两个单点爆左单点
+E：双压</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B690</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：小空白后爆第二个单点（左）
+E：左单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>极限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B688</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左白球
+E：双条</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B429</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左单条后爆白球
+E：左白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B684</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：681左直条按住2cb
+E：左白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A261</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：左直条后爆右单点
+E：双条结束</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A137</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：右手滑球后左直条
+E：左滑+右点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B757</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左点+右条后让左二连点爆右二连点
+E：右单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B728</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左条后爆右点后右条
+E：左二连点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A138</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：一轨单点
+E：二轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B324</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：四轨单点
+E：二轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>爆气</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A85</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：二轨二连点
+E：三轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B598</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：594右手直条按住3cb
+E：左白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B666</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左直条按住1cb
+E：右滑球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B620</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左直条后右手单点
+E：右手白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B356</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左白球
+E：左二连点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A95</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：左白球
+E：左二连点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B348</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：右二连点
+E：左二连点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A142</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：右单点后左单点（压）
+E：右白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A74</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：左手白球
+E：右手白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A96</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：左手二连点
+E：右手二连点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B700</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A148</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：双打后，过小空白爆第二个单点（三轨）（压）
+E：四轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：双打后，过小空白爆第二个单点（二轨）（压）
+E：一轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B836</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：2-1滑键后爆一轨条+4-3滑键
+E：双长条</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A186</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：左直条后右手白球（存）
+E：左单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B243</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：右滑球后左单点
+E：左白球</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A128</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：125右直条按住2cb
+E：右手二连点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B516</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：二轨拐条左滑
+E：2-1滑键</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：一轨拐条右滑
+E：四轨拐条左滑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B433</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：一轨直条按住1cb
+E：一轨直条右滑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A332</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：二轨直条按住1cb
+E：一轨条右滑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B980</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：三轨直条按住2cb
+E：四轨直条左滑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A388</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：二三轨双拐
+E：二轨条</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B772</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：一轨单点
+E：一轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B659</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：653四轨直条按住5cb
+E：4-3滑键</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B744</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：一轨条按住1cb
+E：三轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A169</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：一轨单点
+E：三轨单点（压）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A93</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：三轨单点
+E：二轨直条头</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A134</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：三轨直条按住
+E：四轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B419</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：二轨条
+E：四轨条</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B567</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：三轨条右滑
+E：二轨条左滑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B536</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：二轨条左滑
+E：二轨条</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A384</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：第三组双点
+E：双点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B1276</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：第三组双点
+E：双点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：第三组双点
+E：左滑点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A362</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：左滑点后爆右单点（存）
+E：左单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B689</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：左滑条后右单点
+E：右滑点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B591</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：583右滑条按住7cb
+E：左单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A140</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A：右滑条按住
+E：左滑点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>心上人呀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dream</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Invader</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DEAD OR LIE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B546</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：B开过一组密集乱点后，爆3-4滑键后的第一个四轨单点
+E：三轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：631左手2-1拐条后，爆第四个二轨单点
+E：一轨+四轨双点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>爆气</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B659</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B584</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B：B开过一组密集乱点后，爆3-4滑键、2-1滑键后的第一个单点（三轨）
+E：三轨单点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2984,7 +3473,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3200,10 +3689,16 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规 2" xfId="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3480,8 +3975,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19" style="48" customWidth="1"/>
@@ -3879,21 +4374,37 @@
         <v>298</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" s="56" t="s">
         <v>441</v>
       </c>
       <c r="B13" s="56">
         <v>9</v>
       </c>
-      <c r="C13" s="56"/>
-      <c r="D13" s="56"/>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56"/>
-      <c r="G13" s="56"/>
-      <c r="H13" s="56"/>
-      <c r="I13" s="56"/>
-      <c r="J13" s="56"/>
+      <c r="C13" s="48" t="s">
+        <v>717</v>
+      </c>
+      <c r="D13" s="48" t="s">
+        <v>733</v>
+      </c>
+      <c r="E13" s="56" t="s">
+        <v>731</v>
+      </c>
+      <c r="F13" s="56" t="s">
+        <v>732</v>
+      </c>
+      <c r="G13" s="56" t="s">
+        <v>731</v>
+      </c>
+      <c r="H13" s="56" t="s">
+        <v>679</v>
+      </c>
+      <c r="I13" s="56" t="s">
+        <v>732</v>
+      </c>
+      <c r="J13" s="56">
+        <v>410</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A14" s="56" t="s">
@@ -3959,12 +4470,36 @@
         <v>410</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A16" s="56" t="s">
         <v>453</v>
       </c>
       <c r="B16" s="56">
         <v>6</v>
+      </c>
+      <c r="C16" s="48" t="s">
+        <v>694</v>
+      </c>
+      <c r="D16" s="48" t="s">
+        <v>695</v>
+      </c>
+      <c r="E16" s="48" t="s">
+        <v>696</v>
+      </c>
+      <c r="F16" s="48" t="s">
+        <v>697</v>
+      </c>
+      <c r="G16" s="48" t="s">
+        <v>694</v>
+      </c>
+      <c r="H16" s="48" t="s">
+        <v>698</v>
+      </c>
+      <c r="I16" s="48" t="s">
+        <v>695</v>
+      </c>
+      <c r="J16" s="48">
+        <v>323</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
@@ -4191,37 +4726,69 @@
         <v>750</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A24" s="56" t="s">
         <v>484</v>
       </c>
       <c r="B24" s="56">
         <v>6</v>
       </c>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="56"/>
-      <c r="J24" s="56"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C24" s="56" t="s">
+        <v>754</v>
+      </c>
+      <c r="D24" s="56" t="s">
+        <v>755</v>
+      </c>
+      <c r="E24" s="48" t="s">
+        <v>756</v>
+      </c>
+      <c r="F24" s="48" t="s">
+        <v>757</v>
+      </c>
+      <c r="G24" s="56" t="s">
+        <v>754</v>
+      </c>
+      <c r="H24" s="56" t="s">
+        <v>698</v>
+      </c>
+      <c r="I24" s="56" t="s">
+        <v>755</v>
+      </c>
+      <c r="J24" s="56">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A25" s="56" t="s">
         <v>485</v>
       </c>
       <c r="B25" s="56">
         <v>6</v>
       </c>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="56"/>
-      <c r="J25" s="56"/>
+      <c r="C25" s="56" t="s">
+        <v>744</v>
+      </c>
+      <c r="D25" s="56" t="s">
+        <v>745</v>
+      </c>
+      <c r="E25" s="56" t="s">
+        <v>742</v>
+      </c>
+      <c r="F25" s="56" t="s">
+        <v>743</v>
+      </c>
+      <c r="G25" s="56" t="s">
+        <v>742</v>
+      </c>
+      <c r="H25" s="56" t="s">
+        <v>679</v>
+      </c>
+      <c r="I25" s="56" t="s">
+        <v>743</v>
+      </c>
+      <c r="J25" s="56">
+        <v>372</v>
+      </c>
     </row>
     <row r="26" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A26" s="56" t="s">
@@ -4255,69 +4822,165 @@
         <v>408</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A27" s="56" t="s">
         <v>491</v>
       </c>
       <c r="B27" s="56">
         <v>7</v>
       </c>
-      <c r="C27" s="56"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="56"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="56"/>
-      <c r="H27" s="56"/>
-      <c r="I27" s="56"/>
-      <c r="J27" s="56"/>
-    </row>
-    <row r="28" spans="1:10" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C27" s="48" t="s">
+        <v>750</v>
+      </c>
+      <c r="D27" s="48" t="s">
+        <v>751</v>
+      </c>
+      <c r="E27" s="56" t="s">
+        <v>748</v>
+      </c>
+      <c r="F27" s="56" t="s">
+        <v>749</v>
+      </c>
+      <c r="G27" s="56" t="s">
+        <v>748</v>
+      </c>
+      <c r="H27" s="56" t="s">
+        <v>698</v>
+      </c>
+      <c r="I27" s="56" t="s">
+        <v>749</v>
+      </c>
+      <c r="J27" s="56">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="57" x14ac:dyDescent="0.2">
       <c r="A28" s="56" t="s">
         <v>492</v>
       </c>
       <c r="B28" s="56">
         <v>8</v>
       </c>
-      <c r="C28" s="56"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C28" s="48" t="s">
+        <v>720</v>
+      </c>
+      <c r="D28" s="48" t="s">
+        <v>721</v>
+      </c>
+      <c r="E28" s="56" t="s">
+        <v>719</v>
+      </c>
+      <c r="F28" s="56" t="s">
+        <v>722</v>
+      </c>
+      <c r="G28" s="56" t="s">
+        <v>719</v>
+      </c>
+      <c r="H28" s="56" t="s">
+        <v>679</v>
+      </c>
+      <c r="I28" s="56" t="s">
+        <v>722</v>
+      </c>
+      <c r="J28" s="56">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A29" s="56" t="s">
         <v>493</v>
       </c>
       <c r="B29" s="56">
         <v>8</v>
       </c>
-      <c r="C29" s="56"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="56"/>
-      <c r="J29" s="56"/>
+      <c r="C29" s="56" t="s">
+        <v>736</v>
+      </c>
+      <c r="D29" s="56" t="s">
+        <v>737</v>
+      </c>
+      <c r="E29" s="56" t="s">
+        <v>738</v>
+      </c>
+      <c r="F29" s="56" t="s">
+        <v>739</v>
+      </c>
+      <c r="G29" s="56" t="s">
+        <v>736</v>
+      </c>
+      <c r="H29" s="56" t="s">
+        <v>679</v>
+      </c>
+      <c r="I29" s="56" t="s">
+        <v>737</v>
+      </c>
+      <c r="J29" s="56">
+        <v>623</v>
+      </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="56" t="s">
         <v>494</v>
       </c>
-      <c r="B30" s="56">
+      <c r="B30" s="48">
         <v>10</v>
       </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
-      <c r="I30" s="56"/>
-      <c r="J30" s="56"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" s="48" t="s">
+        <v>773</v>
+      </c>
+      <c r="B31" s="48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" s="48" t="s">
+        <v>774</v>
+      </c>
+      <c r="B32" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A33" s="48" t="s">
+        <v>775</v>
+      </c>
+      <c r="B33" s="48">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>777</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>778</v>
+      </c>
+      <c r="E33" t="s">
+        <v>781</v>
+      </c>
+      <c r="F33" s="23" t="s">
+        <v>779</v>
+      </c>
+      <c r="G33" t="s">
+        <v>781</v>
+      </c>
+      <c r="H33" s="23" t="s">
+        <v>780</v>
+      </c>
+      <c r="I33" s="23" t="s">
+        <v>779</v>
+      </c>
+      <c r="J33">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" s="48" t="s">
+        <v>776</v>
+      </c>
+      <c r="B34" s="48">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -4327,8 +4990,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.375" customWidth="1"/>
@@ -4588,12 +5251,18 @@
       </c>
       <c r="G12" s="48"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>441</v>
       </c>
       <c r="B13" s="59">
         <v>9</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>734</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>735</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
@@ -4636,12 +5305,18 @@
         <v>186</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>453</v>
       </c>
       <c r="B16" s="59">
         <v>6</v>
+      </c>
+      <c r="C16" s="61" t="s">
+        <v>699</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
@@ -4775,20 +5450,32 @@
         <v>186</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A24" s="48" t="s">
         <v>484</v>
       </c>
       <c r="B24" s="48">
         <v>6</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C24" s="23" t="s">
+        <v>758</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A25" s="48" t="s">
         <v>485</v>
       </c>
       <c r="B25" s="48">
         <v>6</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>746</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>747</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
@@ -4811,28 +5498,46 @@
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A27" s="48" t="s">
         <v>491</v>
       </c>
       <c r="B27" s="48">
         <v>7</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C27" s="23" t="s">
+        <v>752</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A28" s="48" t="s">
         <v>492</v>
       </c>
       <c r="B28" s="48">
         <v>8</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C28" t="s">
+        <v>723</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A29" s="57" t="s">
         <v>493</v>
       </c>
       <c r="B29" s="48">
         <v>8</v>
+      </c>
+      <c r="C29" t="s">
+        <v>740</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>741</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="18.75" x14ac:dyDescent="0.2">
@@ -4840,6 +5545,44 @@
         <v>494</v>
       </c>
       <c r="B30" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="48" t="s">
+        <v>773</v>
+      </c>
+      <c r="B31" s="48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="48" t="s">
+        <v>774</v>
+      </c>
+      <c r="B32" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="48" t="s">
+        <v>775</v>
+      </c>
+      <c r="B33" s="48">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>782</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="48" t="s">
+        <v>776</v>
+      </c>
+      <c r="B34" s="48">
         <v>10</v>
       </c>
     </row>
@@ -4851,8 +5594,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.875" customWidth="1"/>
@@ -5120,12 +5863,36 @@
       </c>
       <c r="K8" s="18"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>425</v>
       </c>
       <c r="B9" s="59">
         <v>6</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>709</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>710</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>707</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>708</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>707</v>
+      </c>
+      <c r="H9" s="71" t="s">
+        <v>698</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>708</v>
+      </c>
+      <c r="J9" s="18">
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -5136,12 +5903,36 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>435</v>
       </c>
       <c r="B11" s="59">
         <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>725</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>726</v>
+      </c>
+      <c r="E11" t="s">
+        <v>727</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>728</v>
+      </c>
+      <c r="G11" t="s">
+        <v>727</v>
+      </c>
+      <c r="H11" t="s">
+        <v>698</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>728</v>
+      </c>
+      <c r="J11">
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
@@ -5563,48 +6354,195 @@
         <v>314</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="18.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A25" s="58" t="s">
         <v>486</v>
       </c>
       <c r="B25" s="48">
         <v>7</v>
       </c>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C25" s="23" t="s">
+        <v>701</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>702</v>
+      </c>
+      <c r="E25" t="s">
+        <v>703</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>704</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>701</v>
+      </c>
+      <c r="H25" s="71" t="s">
+        <v>679</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>702</v>
+      </c>
+      <c r="J25">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A26" s="48" t="s">
         <v>491</v>
       </c>
       <c r="B26" s="48">
         <v>7</v>
       </c>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-    </row>
-    <row r="27" spans="1:10" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C26" s="23" t="s">
+        <v>715</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>716</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>713</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>714</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>713</v>
+      </c>
+      <c r="H26" s="71" t="s">
+        <v>698</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>714</v>
+      </c>
+      <c r="J26">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A27" s="48" t="s">
         <v>492</v>
       </c>
       <c r="B27" s="48">
         <v>8</v>
       </c>
-      <c r="C27" s="23"/>
-    </row>
-    <row r="28" spans="1:10" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C27" s="23" t="s">
+        <v>675</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>676</v>
+      </c>
+      <c r="E27" t="s">
+        <v>677</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>678</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>675</v>
+      </c>
+      <c r="H27" s="23" t="s">
+        <v>679</v>
+      </c>
+      <c r="I27" s="23" t="s">
+        <v>676</v>
+      </c>
+      <c r="J27">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A28" s="57" t="s">
         <v>493</v>
       </c>
       <c r="B28" s="48">
         <v>8</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C28" s="23" t="s">
+        <v>682</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="E28" t="s">
+        <v>684</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>685</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>682</v>
+      </c>
+      <c r="H28" s="23" t="s">
+        <v>679</v>
+      </c>
+      <c r="I28" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="J28">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A29" s="57" t="s">
         <v>494</v>
       </c>
       <c r="B29" s="48">
+        <v>10</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>688</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>689</v>
+      </c>
+      <c r="E29" t="s">
+        <v>690</v>
+      </c>
+      <c r="F29" s="23" t="s">
+        <v>691</v>
+      </c>
+      <c r="G29" s="23" t="s">
+        <v>688</v>
+      </c>
+      <c r="H29" s="23" t="s">
+        <v>679</v>
+      </c>
+      <c r="I29" s="23" t="s">
+        <v>689</v>
+      </c>
+      <c r="J29">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" s="48" t="s">
+        <v>773</v>
+      </c>
+      <c r="B30" s="48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" s="48" t="s">
+        <v>774</v>
+      </c>
+      <c r="B31" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" s="48" t="s">
+        <v>775</v>
+      </c>
+      <c r="B32" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="48" t="s">
+        <v>776</v>
+      </c>
+      <c r="B33" s="48">
         <v>10</v>
       </c>
     </row>
@@ -5616,8 +6554,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.125" customWidth="1"/>
@@ -5784,14 +6722,19 @@
         <v>186</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>425</v>
       </c>
       <c r="B9" s="59">
         <v>6</v>
       </c>
-      <c r="C9" s="65"/>
+      <c r="C9" s="65" t="s">
+        <v>711</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>712</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -5802,14 +6745,19 @@
       </c>
       <c r="C10" s="65"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>435</v>
       </c>
       <c r="B11" s="59">
         <v>6</v>
       </c>
-      <c r="C11" s="65"/>
+      <c r="C11" s="65" t="s">
+        <v>729</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>730</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -6083,50 +7031,107 @@
         <v>186</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="18.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A25" s="58" t="s">
         <v>486</v>
       </c>
       <c r="B25" s="48">
         <v>7</v>
       </c>
-      <c r="C25" s="23"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C25" s="23" t="s">
+        <v>705</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A26" s="48" t="s">
         <v>491</v>
       </c>
       <c r="B26" s="48">
         <v>7</v>
       </c>
-      <c r="C26" s="23"/>
-    </row>
-    <row r="27" spans="1:7" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C26" s="23" t="s">
+        <v>717</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A27" s="48" t="s">
         <v>492</v>
       </c>
       <c r="B27" s="48">
         <v>8</v>
       </c>
-      <c r="C27" s="23"/>
-    </row>
-    <row r="28" spans="1:7" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C27" s="23" t="s">
+        <v>680</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A28" s="57" t="s">
         <v>493</v>
       </c>
       <c r="B28" s="48">
         <v>8</v>
       </c>
-      <c r="C28" s="65"/>
-    </row>
-    <row r="29" spans="1:7" ht="18.75" x14ac:dyDescent="0.2">
+      <c r="C28" s="65" t="s">
+        <v>686</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A29" s="57" t="s">
         <v>494</v>
       </c>
       <c r="B29" s="48">
         <v>10</v>
       </c>
-      <c r="C29" s="65"/>
+      <c r="C29" s="65" t="s">
+        <v>692</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="48" t="s">
+        <v>773</v>
+      </c>
+      <c r="B30" s="48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="48" t="s">
+        <v>774</v>
+      </c>
+      <c r="B31" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="48" t="s">
+        <v>775</v>
+      </c>
+      <c r="B32" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="48" t="s">
+        <v>776</v>
+      </c>
+      <c r="B33" s="48">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -6135,8 +7140,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K24"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.875" customWidth="1"/>
@@ -6722,23 +7727,69 @@
         <v>654</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A19" s="65" t="s">
         <v>478</v>
       </c>
       <c r="B19" s="59">
         <v>10</v>
       </c>
-      <c r="H19" s="23"/>
-    </row>
-    <row r="20" spans="1:10" ht="33" x14ac:dyDescent="0.2">
+      <c r="C19" s="61" t="s">
+        <v>760</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>761</v>
+      </c>
+      <c r="E19" t="s">
+        <v>762</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>763</v>
+      </c>
+      <c r="G19" s="61" t="s">
+        <v>760</v>
+      </c>
+      <c r="H19" s="23" t="s">
+        <v>446</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>761</v>
+      </c>
+      <c r="J19" s="72">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A20" s="69" t="s">
         <v>486</v>
       </c>
       <c r="B20" s="48">
         <v>6</v>
       </c>
-      <c r="H20" s="23"/>
+      <c r="C20" s="61" t="s">
+        <v>765</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>766</v>
+      </c>
+      <c r="E20" t="s">
+        <v>769</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>770</v>
+      </c>
+      <c r="G20" s="61" t="s">
+        <v>771</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>679</v>
+      </c>
+      <c r="I20" s="23" t="s">
+        <v>772</v>
+      </c>
+      <c r="J20" s="72">
+        <v>401</v>
+      </c>
     </row>
     <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.2">
       <c r="A21" s="56" t="s">
@@ -6769,7 +7820,7 @@
         <v>634</v>
       </c>
       <c r="J21">
-        <v>466</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
@@ -6848,15 +7899,40 @@
       <c r="H24" s="23"/>
       <c r="I24" s="23"/>
     </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="48" t="s">
+        <v>774</v>
+      </c>
+      <c r="B25" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="48" t="s">
+        <v>775</v>
+      </c>
+      <c r="B26" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="48" t="s">
+        <v>776</v>
+      </c>
+      <c r="B27" s="48">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G24"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.25" style="23" customWidth="1"/>
@@ -7238,23 +8314,35 @@
         <v>186</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>478</v>
       </c>
       <c r="B19" s="59">
         <v>10</v>
       </c>
+      <c r="C19" s="61" t="s">
+        <v>760</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>764</v>
+      </c>
       <c r="F19" s="53" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A20" s="58" t="s">
         <v>486</v>
       </c>
       <c r="B20" s="48">
         <v>6</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>767</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>768</v>
       </c>
       <c r="F20" s="53" t="s">
         <v>186</v>
@@ -7274,7 +8362,7 @@
         <v>647</v>
       </c>
       <c r="E21" s="23">
-        <v>466</v>
+        <v>224</v>
       </c>
       <c r="F21" s="53" t="s">
         <v>186</v>
@@ -7326,6 +8414,30 @@
       </c>
       <c r="F24" s="53" t="s">
         <v>186</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="48" t="s">
+        <v>774</v>
+      </c>
+      <c r="B25" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="48" t="s">
+        <v>775</v>
+      </c>
+      <c r="B26" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="48" t="s">
+        <v>776</v>
+      </c>
+      <c r="B27" s="48">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -7335,7 +8447,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -8480,7 +9592,7 @@
     <row r="40" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="41" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A1:M41">
+  <autoFilter ref="A1:M41" xr:uid="{00000000-0009-0000-0000-000006000000}">
     <filterColumn colId="1">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -8494,7 +9606,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>